<commit_message>
Atualiza lista de operadores
</commit_message>
<xml_diff>
--- a/LISTA DE OPERADORES.xlsx
+++ b/LISTA DE OPERADORES.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\PROJETOS EM ANDAMENTO\PAINEL DE CONTROLE MTECH\PROGRAMAS\PROJETOS -BACKEND\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\PROJETOS EM ANDAMENTO\PAINEL DE CONTROLE MTECH\PROGRAMAS\PROJETOS---BACKEND-IA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AA9D96B-B7AD-4627-82C0-AF52F011AA5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B86F694-CF39-48F2-BEF3-173B1EB35F2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{AC9FE68F-77C9-4D03-9827-DD98DE9BB2CF}"/>
+    <workbookView xWindow="585" yWindow="5085" windowWidth="38700" windowHeight="15345" xr2:uid="{AC9FE68F-77C9-4D03-9827-DD98DE9BB2CF}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>VANILDO ROCHA FRANCO</t>
   </si>
@@ -150,6 +150,9 @@
   </si>
   <si>
     <t>HIAGO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAULO </t>
   </si>
 </sst>
 </file>
@@ -220,8 +223,8 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -556,7 +559,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AA4E20E-2919-4396-A145-A937C26D729E}">
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:A38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.85546875" bestFit="1" customWidth="1"/>
@@ -634,7 +637,7 @@
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -699,58 +702,63 @@
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>25</v>
+      <c r="A28" s="3" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>8</v>
+        <v>26</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A37">
-    <sortCondition ref="A1:A37"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A38">
+    <sortCondition ref="A16:A38"/>
   </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>